<commit_message>
docs: add system architecture, agent system deep dive, rebuild specification, and update codebase
</commit_message>
<xml_diff>
--- a/ai-governance-main/backend/Agents/predefined_controls.xlsx
+++ b/ai-governance-main/backend/Agents/predefined_controls.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jhanakshukla/Desktop/rakfort ai governance/governance-agents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pranay Gupta\Pictures\AI-Goverance-Health\ai-governance-main\backend\Agents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0112CD46-35E5-6C4A-906D-6E9BD75CC827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{342B50FA-A7B6-4633-87B5-286664282C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -838,14 +838,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="2" max="2" width="39.21875" customWidth="1"/>
+    <col min="3" max="3" width="42.77734375" customWidth="1"/>
     <col min="4" max="4" width="116.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -859,7 +859,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -873,7 +873,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -887,7 +887,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -901,7 +901,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -915,7 +915,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -929,7 +929,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -943,7 +943,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -957,7 +957,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -971,7 +971,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -985,7 +985,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -999,7 +999,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1041,7 +1041,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -1139,7 +1139,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -1167,7 +1167,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -1195,7 +1195,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>29</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -1237,7 +1237,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>31</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>32</v>
       </c>
@@ -1265,7 +1265,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>33</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>34</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>35</v>
       </c>
@@ -1307,7 +1307,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>36</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>38</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>39</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>40</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>41</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>42</v>
       </c>
@@ -1405,7 +1405,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>43</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>44</v>
       </c>
@@ -1433,7 +1433,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>46</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>47</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>48</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>49</v>
       </c>

</xml_diff>